<commit_message>
Add SALT_CLOTHES_KONKURS_1210.xlsx: non-auction salt/clothing lots with deadline from 16.10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/SALT_CLOTHES_1210.xlsx
+++ b/SALT_CLOTHES_1210.xlsx
@@ -888,7 +888,11 @@
           <t>открыть</t>
         </is>
       </c>
-      <c r="R5" s="7" t="inlineStr"/>
+      <c r="R5" s="7" t="inlineStr">
+        <is>
+          <t>в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1454,7 +1458,7 @@
       <c r="Q14" s="12" t="inlineStr"/>
       <c r="R14" s="12" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1999,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2063,7 @@
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2127,7 @@
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2183,7 @@
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2247,7 @@
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2311,7 @@
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2463,7 @@
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>крупный лот &gt;50 млн</t>
+          <t>крупный лот &gt;50 млн; в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2537,7 @@
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>крупный лот &gt;50 млн</t>
+          <t>крупный лот &gt;50 млн; в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2959,11 @@
           <t>открыть</t>
         </is>
       </c>
-      <c r="R21" s="7" t="inlineStr"/>
+      <c r="R21" s="7" t="inlineStr">
+        <is>
+          <t>в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -3089,7 +3097,11 @@
           <t>открыть</t>
         </is>
       </c>
-      <c r="R23" s="7" t="inlineStr"/>
+      <c r="R23" s="7" t="inlineStr">
+        <is>
+          <t>в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -3225,7 +3237,11 @@
           <t>открыть</t>
         </is>
       </c>
-      <c r="R25" s="7" t="inlineStr"/>
+      <c r="R25" s="7" t="inlineStr">
+        <is>
+          <t>в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -4133,7 +4149,11 @@
           <t>открыть</t>
         </is>
       </c>
-      <c r="R38" s="7" t="inlineStr"/>
+      <c r="R38" s="7" t="inlineStr">
+        <is>
+          <t>в ЕИС «иной способ» — уточнить в извещении (не аукцион)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -4545,7 +4565,7 @@
       <c r="Q44" s="7" t="inlineStr"/>
       <c r="R44" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4629,7 @@
       <c r="Q45" s="7" t="inlineStr"/>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4697,7 @@
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4761,7 @@
       <c r="Q47" s="7" t="inlineStr"/>
       <c r="R47" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4825,7 @@
       <c r="Q48" s="7" t="inlineStr"/>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4885,7 @@
       <c r="Q49" s="7" t="inlineStr"/>
       <c r="R49" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4949,7 @@
       <c r="Q50" s="7" t="inlineStr"/>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -4993,7 +5013,7 @@
       <c r="Q51" s="7" t="inlineStr"/>
       <c r="R51" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5077,7 @@
       <c r="Q52" s="7" t="inlineStr"/>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5141,7 @@
       <c r="Q53" s="7" t="inlineStr"/>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5209,7 @@
       </c>
       <c r="R54" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5273,7 @@
       <c r="Q55" s="7" t="inlineStr"/>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5337,7 @@
       <c r="Q56" s="7" t="inlineStr"/>
       <c r="R56" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5401,7 @@
       <c r="Q57" s="7" t="inlineStr"/>
       <c r="R57" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5445,7 +5465,7 @@
       <c r="Q58" s="7" t="inlineStr"/>
       <c r="R58" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5513,7 +5533,7 @@
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5577,7 +5597,7 @@
       <c r="Q60" s="7" t="inlineStr"/>
       <c r="R60" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5661,7 @@
       <c r="Q61" s="7" t="inlineStr"/>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5705,7 +5725,7 @@
       <c r="Q62" s="7" t="inlineStr"/>
       <c r="R62" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5769,7 +5789,7 @@
       <c r="Q63" s="7" t="inlineStr"/>
       <c r="R63" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5853,7 @@
       <c r="Q64" s="7" t="inlineStr"/>
       <c r="R64" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5917,7 @@
       <c r="Q65" s="7" t="inlineStr"/>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6167,7 @@
       <c r="Q69" s="12" t="inlineStr"/>
       <c r="R69" s="12" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -6203,7 +6223,7 @@
       <c r="Q70" s="12" t="inlineStr"/>
       <c r="R70" s="12" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6287,7 @@
       <c r="Q71" s="12" t="inlineStr"/>
       <c r="R71" s="12" t="inlineStr">
         <is>
-          <t>НМЦК не указана — коммерческая, цену запрашивать</t>
+          <t>НМЦК не указана — цену запрашивать</t>
         </is>
       </c>
     </row>

</xml_diff>